<commit_message>
added gpio funcionalities, buttons, sw2 and buzzer
</commit_message>
<xml_diff>
--- a/docs/Hiwonder Board V1.2/Pinout list.xlsx
+++ b/docs/Hiwonder Board V1.2/Pinout list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\sme\sme-stm32f407-4wcl\docs\Hiwonder Board V1.2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE5C97A6-234D-472B-8B6E-E2401A69EA88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C206DB1-E99B-474A-B967-791054AE5EA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5051D413-03F4-420B-86D3-BBB2B92BD681}"/>
+    <workbookView xWindow="-120" yWindow="16080" windowWidth="29040" windowHeight="15720" xr2:uid="{5051D413-03F4-420B-86D3-BBB2B92BD681}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="167">
   <si>
     <t>PE10</t>
   </si>
@@ -107,12 +107,6 @@
     <t>K2</t>
   </si>
   <si>
-    <t>K1_BUTTON</t>
-  </si>
-  <si>
-    <t>K2_BUTTON</t>
-  </si>
-  <si>
     <t>PE7</t>
   </si>
   <si>
@@ -534,6 +528,15 @@
   </si>
   <si>
     <t>USB Host Data Minus (D-)</t>
+  </si>
+  <si>
+    <t>USER_SW3</t>
+  </si>
+  <si>
+    <t>USER_K1_BUTTON</t>
+  </si>
+  <si>
+    <t>USER_K2_BUTTON</t>
   </si>
 </sst>
 </file>
@@ -935,30 +938,30 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D1" t="s">
         <v>18</v>
       </c>
       <c r="E1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
@@ -970,18 +973,18 @@
         <v>5</v>
       </c>
       <c r="E2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B3" t="s">
         <v>1</v>
@@ -993,18 +996,18 @@
         <v>3</v>
       </c>
       <c r="E3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G3" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
@@ -1016,18 +1019,18 @@
         <v>4</v>
       </c>
       <c r="E4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G4" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B5" t="s">
         <v>7</v>
@@ -1039,18 +1042,18 @@
         <v>9</v>
       </c>
       <c r="E5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F5" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G5" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
@@ -1062,13 +1065,13 @@
         <v>10</v>
       </c>
       <c r="E6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G6" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1085,18 +1088,18 @@
         <v>14</v>
       </c>
       <c r="E7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F7" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G7" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B8" t="s">
         <v>16</v>
@@ -1105,21 +1108,21 @@
         <v>17</v>
       </c>
       <c r="D8" t="s">
-        <v>17</v>
+        <v>164</v>
       </c>
       <c r="E8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G8" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B9" t="s">
         <v>19</v>
@@ -1128,21 +1131,21 @@
         <v>21</v>
       </c>
       <c r="D9" t="s">
-        <v>23</v>
+        <v>165</v>
       </c>
       <c r="E9" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F9" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G9" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B10" t="s">
         <v>20</v>
@@ -1151,729 +1154,729 @@
         <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
+        <v>166</v>
       </c>
       <c r="E10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F10" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G10" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E11" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F11" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G11" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D12" t="s">
         <v>36</v>
       </c>
-      <c r="B12" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" t="s">
-        <v>69</v>
-      </c>
-      <c r="D12" t="s">
-        <v>38</v>
-      </c>
       <c r="E12" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F12" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G12" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E13" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F13" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G13" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C14" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E14" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F14" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G14" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" t="s">
+        <v>92</v>
+      </c>
+      <c r="D15" t="s">
+        <v>43</v>
+      </c>
+      <c r="E15" t="s">
         <v>44</v>
       </c>
-      <c r="C15" t="s">
-        <v>94</v>
-      </c>
-      <c r="D15" t="s">
-        <v>45</v>
-      </c>
-      <c r="E15" t="s">
-        <v>46</v>
-      </c>
       <c r="F15" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G15" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" t="s">
+        <v>92</v>
+      </c>
+      <c r="D16" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" t="s">
         <v>47</v>
       </c>
-      <c r="C16" t="s">
-        <v>94</v>
-      </c>
-      <c r="D16" t="s">
-        <v>48</v>
-      </c>
-      <c r="E16" t="s">
-        <v>49</v>
-      </c>
       <c r="F16" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G16" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C17" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D17" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E17" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F17" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="G17" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C18" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D18" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E18" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F18" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="G18" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B19" t="s">
+        <v>54</v>
+      </c>
+      <c r="C19" t="s">
+        <v>106</v>
+      </c>
+      <c r="D19" t="s">
+        <v>55</v>
+      </c>
+      <c r="E19" t="s">
         <v>56</v>
       </c>
-      <c r="C19" t="s">
-        <v>108</v>
-      </c>
-      <c r="D19" t="s">
-        <v>57</v>
-      </c>
-      <c r="E19" t="s">
-        <v>58</v>
-      </c>
       <c r="F19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G19" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B20" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" t="s">
+        <v>106</v>
+      </c>
+      <c r="D20" t="s">
+        <v>58</v>
+      </c>
+      <c r="E20" t="s">
         <v>59</v>
       </c>
-      <c r="C20" t="s">
-        <v>108</v>
-      </c>
-      <c r="D20" t="s">
-        <v>60</v>
-      </c>
-      <c r="E20" t="s">
-        <v>61</v>
-      </c>
       <c r="F20" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G20" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B21" t="s">
+        <v>60</v>
+      </c>
+      <c r="C21" t="s">
+        <v>113</v>
+      </c>
+      <c r="D21" t="s">
+        <v>61</v>
+      </c>
+      <c r="E21" t="s">
         <v>62</v>
       </c>
-      <c r="C21" t="s">
-        <v>115</v>
-      </c>
-      <c r="D21" t="s">
-        <v>63</v>
-      </c>
-      <c r="E21" t="s">
-        <v>64</v>
-      </c>
       <c r="F21" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G21" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C22" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E22" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F22" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G22" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B23" t="s">
+        <v>89</v>
+      </c>
+      <c r="C23" t="s">
+        <v>92</v>
+      </c>
+      <c r="D23" t="s">
+        <v>90</v>
+      </c>
+      <c r="E23" t="s">
         <v>91</v>
       </c>
-      <c r="C23" t="s">
-        <v>94</v>
-      </c>
-      <c r="D23" t="s">
-        <v>92</v>
-      </c>
-      <c r="E23" t="s">
-        <v>93</v>
-      </c>
       <c r="F23" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G23" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B24" t="s">
+        <v>93</v>
+      </c>
+      <c r="C24" t="s">
+        <v>92</v>
+      </c>
+      <c r="D24" t="s">
+        <v>94</v>
+      </c>
+      <c r="E24" t="s">
         <v>95</v>
       </c>
-      <c r="C24" t="s">
-        <v>94</v>
-      </c>
-      <c r="D24" t="s">
-        <v>96</v>
-      </c>
-      <c r="E24" t="s">
-        <v>97</v>
-      </c>
       <c r="F24" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G24" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B25" t="s">
+        <v>96</v>
+      </c>
+      <c r="C25" t="s">
+        <v>99</v>
+      </c>
+      <c r="D25" t="s">
+        <v>97</v>
+      </c>
+      <c r="E25" t="s">
         <v>98</v>
       </c>
-      <c r="C25" t="s">
-        <v>101</v>
-      </c>
-      <c r="D25" t="s">
-        <v>99</v>
-      </c>
-      <c r="E25" t="s">
-        <v>100</v>
-      </c>
       <c r="F25" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G25" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B26" t="s">
+        <v>100</v>
+      </c>
+      <c r="C26" t="s">
+        <v>99</v>
+      </c>
+      <c r="D26" t="s">
+        <v>101</v>
+      </c>
+      <c r="E26" t="s">
         <v>102</v>
       </c>
-      <c r="C26" t="s">
-        <v>101</v>
-      </c>
-      <c r="D26" t="s">
-        <v>103</v>
-      </c>
-      <c r="E26" t="s">
-        <v>104</v>
-      </c>
       <c r="F26" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G26" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B27" t="s">
+        <v>103</v>
+      </c>
+      <c r="C27" t="s">
+        <v>106</v>
+      </c>
+      <c r="D27" t="s">
+        <v>104</v>
+      </c>
+      <c r="E27" t="s">
         <v>105</v>
       </c>
-      <c r="C27" t="s">
-        <v>108</v>
-      </c>
-      <c r="D27" t="s">
-        <v>106</v>
-      </c>
-      <c r="E27" t="s">
-        <v>107</v>
-      </c>
       <c r="F27" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G27" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B28" t="s">
+        <v>107</v>
+      </c>
+      <c r="C28" t="s">
+        <v>106</v>
+      </c>
+      <c r="D28" t="s">
+        <v>108</v>
+      </c>
+      <c r="E28" t="s">
         <v>109</v>
       </c>
-      <c r="C28" t="s">
-        <v>108</v>
-      </c>
-      <c r="D28" t="s">
-        <v>110</v>
-      </c>
-      <c r="E28" t="s">
-        <v>111</v>
-      </c>
       <c r="F28" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G28" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B29" t="s">
+        <v>110</v>
+      </c>
+      <c r="C29" t="s">
+        <v>113</v>
+      </c>
+      <c r="D29" t="s">
+        <v>111</v>
+      </c>
+      <c r="E29" t="s">
         <v>112</v>
       </c>
-      <c r="C29" t="s">
-        <v>115</v>
-      </c>
-      <c r="D29" t="s">
-        <v>113</v>
-      </c>
-      <c r="E29" t="s">
-        <v>114</v>
-      </c>
       <c r="F29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G29" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B30" t="s">
+        <v>114</v>
+      </c>
+      <c r="C30" t="s">
+        <v>113</v>
+      </c>
+      <c r="D30" t="s">
+        <v>115</v>
+      </c>
+      <c r="E30" t="s">
         <v>116</v>
       </c>
-      <c r="C30" t="s">
-        <v>115</v>
-      </c>
-      <c r="D30" t="s">
-        <v>117</v>
-      </c>
-      <c r="E30" t="s">
-        <v>118</v>
-      </c>
       <c r="F30" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G30" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>117</v>
+      </c>
+      <c r="B31" t="s">
+        <v>88</v>
+      </c>
+      <c r="C31" t="s">
+        <v>78</v>
+      </c>
+      <c r="D31" t="s">
+        <v>120</v>
+      </c>
+      <c r="E31" t="s">
         <v>119</v>
       </c>
-      <c r="B31" t="s">
-        <v>90</v>
-      </c>
-      <c r="C31" t="s">
-        <v>80</v>
-      </c>
-      <c r="D31" t="s">
-        <v>122</v>
-      </c>
-      <c r="E31" t="s">
-        <v>121</v>
-      </c>
       <c r="F31" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="G31" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B32" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C32" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D32" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E32" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F32" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="G32" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B33" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C33" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D33" t="s">
+        <v>125</v>
+      </c>
+      <c r="E33" t="s">
+        <v>129</v>
+      </c>
+      <c r="F33" t="s">
         <v>127</v>
       </c>
-      <c r="E33" t="s">
-        <v>131</v>
-      </c>
-      <c r="F33" t="s">
-        <v>129</v>
-      </c>
       <c r="G33" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>121</v>
+      </c>
+      <c r="B34" t="s">
         <v>123</v>
       </c>
-      <c r="B34" t="s">
-        <v>125</v>
-      </c>
       <c r="C34" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D34" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E34" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F34" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="G34" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>150</v>
+      </c>
+      <c r="B35" t="s">
+        <v>131</v>
+      </c>
+      <c r="C35" t="s">
+        <v>132</v>
+      </c>
+      <c r="D35" t="s">
+        <v>151</v>
+      </c>
+      <c r="E35" t="s">
         <v>152</v>
       </c>
-      <c r="B35" t="s">
-        <v>133</v>
-      </c>
-      <c r="C35" t="s">
-        <v>134</v>
-      </c>
-      <c r="D35" t="s">
+      <c r="F35" t="s">
         <v>153</v>
       </c>
-      <c r="E35" t="s">
-        <v>154</v>
-      </c>
-      <c r="F35" t="s">
-        <v>155</v>
-      </c>
       <c r="G35" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B36" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C36" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D36" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E36" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F36" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G36" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>141</v>
+      </c>
+      <c r="B37" t="s">
+        <v>139</v>
+      </c>
+      <c r="C37" t="s">
+        <v>134</v>
+      </c>
+      <c r="D37" t="s">
         <v>143</v>
       </c>
-      <c r="B37" t="s">
-        <v>141</v>
-      </c>
-      <c r="C37" t="s">
-        <v>136</v>
-      </c>
-      <c r="D37" t="s">
-        <v>145</v>
-      </c>
       <c r="E37" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F37" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G37" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B38" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C38" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D38" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E38" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F38" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G38" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B39" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C39" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D39" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E39" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F39" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G39" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>156</v>
+      </c>
+      <c r="B40" t="s">
         <v>158</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
+        <v>157</v>
+      </c>
+      <c r="D40" t="s">
         <v>160</v>
       </c>
-      <c r="C40" t="s">
-        <v>159</v>
-      </c>
-      <c r="D40" t="s">
+      <c r="E40" t="s">
         <v>162</v>
       </c>
-      <c r="E40" t="s">
-        <v>164</v>
-      </c>
       <c r="F40" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G40" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B41" t="s">
+        <v>159</v>
+      </c>
+      <c r="C41" t="s">
+        <v>157</v>
+      </c>
+      <c r="D41" t="s">
         <v>161</v>
       </c>
-      <c r="C41" t="s">
-        <v>159</v>
-      </c>
-      <c r="D41" t="s">
+      <c r="E41" t="s">
         <v>163</v>
       </c>
-      <c r="E41" t="s">
-        <v>165</v>
-      </c>
       <c r="F41" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G41" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
implement new arquitecture to send data add missing peripherals
</commit_message>
<xml_diff>
--- a/docs/Hiwonder Board V1.2/Pinout list.xlsx
+++ b/docs/Hiwonder Board V1.2/Pinout list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\sme\sme-stm32f407-4wcl\docs\Hiwonder Board V1.2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F332A49-1F11-4198-A846-37FCBC96620B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DCB16EA-7629-44F9-89A0-624B63FB7D54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="16080" windowWidth="29040" windowHeight="15720" xr2:uid="{5051D413-03F4-420B-86D3-BBB2B92BD681}"/>
   </bookViews>
@@ -143,12 +143,6 @@
     <t>SERVO</t>
   </si>
   <si>
-    <t>PC6_TX</t>
-  </si>
-  <si>
-    <t>PC7_RX</t>
-  </si>
-  <si>
     <t>MOTORS</t>
   </si>
   <si>
@@ -275,9 +269,6 @@
     <t>PA0</t>
   </si>
   <si>
-    <t>ENC1_PHASE_A</t>
-  </si>
-  <si>
     <t>Encoder Motor 1 Phase A</t>
   </si>
   <si>
@@ -287,18 +278,12 @@
     <t>PA1</t>
   </si>
   <si>
-    <t>ENC1_PHASE_B</t>
-  </si>
-  <si>
     <t>Encoder Motor 1 Phase B</t>
   </si>
   <si>
     <t>PA15</t>
   </si>
   <si>
-    <t>ENC2_PHASE_A</t>
-  </si>
-  <si>
     <t>Encoder Motor 2 Phase A</t>
   </si>
   <si>
@@ -308,18 +293,12 @@
     <t>PB3</t>
   </si>
   <si>
-    <t>ENC2_PHASE_B</t>
-  </si>
-  <si>
     <t>Encoder Motor 2 Phase B</t>
   </si>
   <si>
     <t>PB6</t>
   </si>
   <si>
-    <t>ENC3_PHASE_A</t>
-  </si>
-  <si>
     <t>Encoder Motor 3 Phase A</t>
   </si>
   <si>
@@ -329,18 +308,12 @@
     <t>PB7</t>
   </si>
   <si>
-    <t>ENC3_PHASE_B</t>
-  </si>
-  <si>
     <t>Encoder Motor 3 Phase B</t>
   </si>
   <si>
     <t>PB4</t>
   </si>
   <si>
-    <t>ENC4_PHASE_A</t>
-  </si>
-  <si>
     <t>Encoder Motor 4 Phase A</t>
   </si>
   <si>
@@ -350,9 +323,6 @@
     <t>PB5</t>
   </si>
   <si>
-    <t>ENC4_PHASE_B</t>
-  </si>
-  <si>
     <t>Encoder Motor 4 Phase B</t>
   </si>
   <si>
@@ -540,6 +510,36 @@
   </si>
   <si>
     <t xml:space="preserve">Control UART RX from Servo </t>
+  </si>
+  <si>
+    <t>SERIAL_SERVO_UART6_RX</t>
+  </si>
+  <si>
+    <t>SERIAL_SERVO_UART6_TX</t>
+  </si>
+  <si>
+    <t>ENC1_A_TIM5_CH1</t>
+  </si>
+  <si>
+    <t>ENC2_A_TIM2_CH1</t>
+  </si>
+  <si>
+    <t>ENC2_B_TIM2_CH2</t>
+  </si>
+  <si>
+    <t>ENC1_B_TIM5_CH2</t>
+  </si>
+  <si>
+    <t>ENC3_A_TIM4_CH1</t>
+  </si>
+  <si>
+    <t>ENC3_B_TIM4_CH2</t>
+  </si>
+  <si>
+    <t>ENC4_B_TIM3_CH2</t>
+  </si>
+  <si>
+    <t>ENC4_A_TIM3_CH1</t>
   </si>
 </sst>
 </file>
@@ -941,13 +941,13 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D1" t="s">
         <v>18</v>
@@ -956,10 +956,10 @@
         <v>27</v>
       </c>
       <c r="F1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G1" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -979,10 +979,10 @@
         <v>28</v>
       </c>
       <c r="F2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G2" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -999,13 +999,13 @@
         <v>3</v>
       </c>
       <c r="E3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="G3" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1022,13 +1022,13 @@
         <v>4</v>
       </c>
       <c r="E4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F4" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="G4" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1045,13 +1045,13 @@
         <v>9</v>
       </c>
       <c r="E5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G5" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1068,13 +1068,13 @@
         <v>10</v>
       </c>
       <c r="E6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G6" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1091,13 +1091,13 @@
         <v>14</v>
       </c>
       <c r="E7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G7" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1111,16 +1111,16 @@
         <v>17</v>
       </c>
       <c r="D8" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="E8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G8" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1134,16 +1134,16 @@
         <v>21</v>
       </c>
       <c r="D9" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="E9" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F9" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G9" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1157,16 +1157,16 @@
         <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="E10" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F10" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G10" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1177,19 +1177,19 @@
         <v>24</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D11" t="s">
-        <v>35</v>
+        <v>159</v>
       </c>
       <c r="E11" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F11" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G11" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1200,19 +1200,19 @@
         <v>25</v>
       </c>
       <c r="C12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D12" t="s">
-        <v>36</v>
+        <v>158</v>
       </c>
       <c r="E12" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F12" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G12" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1223,19 +1223,19 @@
         <v>26</v>
       </c>
       <c r="C13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D13" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="E13" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="F13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G13" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1246,640 +1246,640 @@
         <v>23</v>
       </c>
       <c r="C14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D14" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="E14" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G14" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C15" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D15" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="E15" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G15" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B16" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C16" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D16" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="E16" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G16" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B17" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C17" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D17" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="E17" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F17" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G17" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B18" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C18" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D18" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="E18" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F18" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G18" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C19" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="D19" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="E19" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F19" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G19" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C20" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="D20" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="E20" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F20" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G20" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B21" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C21" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="D21" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="E21" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F21" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G21" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B22" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C22" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="D22" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="E22" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F22" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G22" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B23" t="s">
+        <v>76</v>
+      </c>
+      <c r="C23" t="s">
         <v>78</v>
       </c>
-      <c r="C23" t="s">
-        <v>81</v>
-      </c>
       <c r="D23" t="s">
-        <v>79</v>
+        <v>160</v>
       </c>
       <c r="E23" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F23" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G23" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B24" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C24" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D24" t="s">
-        <v>83</v>
+        <v>163</v>
       </c>
       <c r="E24" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F24" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G24" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C25" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D25" t="s">
-        <v>86</v>
+        <v>161</v>
       </c>
       <c r="E25" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="F25" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G25" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C26" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D26" t="s">
-        <v>90</v>
+        <v>162</v>
       </c>
       <c r="E26" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="F26" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G26" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B27" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="C27" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="D27" t="s">
-        <v>93</v>
+        <v>164</v>
       </c>
       <c r="E27" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="F27" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G27" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B28" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="C28" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="D28" t="s">
-        <v>97</v>
+        <v>165</v>
       </c>
       <c r="E28" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="F28" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G28" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B29" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C29" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="D29" t="s">
-        <v>100</v>
+        <v>167</v>
       </c>
       <c r="E29" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="F29" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G29" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B30" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="C30" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="D30" t="s">
-        <v>104</v>
+        <v>166</v>
       </c>
       <c r="E30" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="F30" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G30" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B31" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C31" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D31" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="E31" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="F31" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="G31" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="B32" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C32" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D32" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="E32" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="F32" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="G32" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="B33" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="C33" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D33" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="E33" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="F33" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="G33" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="B34" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="C34" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D34" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="E34" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="F34" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="G34" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="B35" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="C35" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="D35" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="E35" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="F35" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="G35" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="B36" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="C36" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="D36" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="E36" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="F36" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G36" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="B37" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="C37" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="D37" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="E37" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="F37" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G37" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="B38" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="C38" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="D38" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="E38" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="F38" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G38" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="B39" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="C39" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="D39" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="E39" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="F39" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G39" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="B40" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="C40" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="D40" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="E40" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="F40" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G40" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="B41" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="C41" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="D41" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="E41" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="F41" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G41" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: gmaepad joy functionality
</commit_message>
<xml_diff>
--- a/docs/Hiwonder Board V1.2/Pinout list.xlsx
+++ b/docs/Hiwonder Board V1.2/Pinout list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\sme\sme-stm32f407-4wcl\docs\Hiwonder Board V1.2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DCB16EA-7629-44F9-89A0-624B63FB7D54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBB2E1DC-2010-45C2-B740-763A818CB593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="16080" windowWidth="29040" windowHeight="15720" xr2:uid="{5051D413-03F4-420B-86D3-BBB2B92BD681}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5051D413-03F4-420B-86D3-BBB2B92BD681}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -1281,7 +1281,7 @@
         <v>69</v>
       </c>
       <c r="G15" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1304,7 +1304,7 @@
         <v>69</v>
       </c>
       <c r="G16" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1327,7 +1327,7 @@
         <v>70</v>
       </c>
       <c r="G17" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1350,7 +1350,7 @@
         <v>70</v>
       </c>
       <c r="G18" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1373,7 +1373,7 @@
         <v>68</v>
       </c>
       <c r="G19" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -1396,7 +1396,7 @@
         <v>68</v>
       </c>
       <c r="G20" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -1419,7 +1419,7 @@
         <v>67</v>
       </c>
       <c r="G21" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -1442,7 +1442,7 @@
         <v>67</v>
       </c>
       <c r="G22" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -1465,7 +1465,7 @@
         <v>65</v>
       </c>
       <c r="G23" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -1488,7 +1488,7 @@
         <v>65</v>
       </c>
       <c r="G24" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -1511,7 +1511,7 @@
         <v>65</v>
       </c>
       <c r="G25" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -1534,7 +1534,7 @@
         <v>65</v>
       </c>
       <c r="G26" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -1557,7 +1557,7 @@
         <v>65</v>
       </c>
       <c r="G27" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -1580,7 +1580,7 @@
         <v>65</v>
       </c>
       <c r="G28" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -1603,7 +1603,7 @@
         <v>65</v>
       </c>
       <c r="G29" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -1626,7 +1626,7 @@
         <v>65</v>
       </c>
       <c r="G30" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -1672,7 +1672,7 @@
         <v>106</v>
       </c>
       <c r="G32" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
@@ -1695,7 +1695,7 @@
         <v>106</v>
       </c>
       <c r="G33" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -1718,7 +1718,7 @@
         <v>106</v>
       </c>
       <c r="G34" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
@@ -1856,7 +1856,7 @@
         <v>65</v>
       </c>
       <c r="G40" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
@@ -1879,7 +1879,7 @@
         <v>65</v>
       </c>
       <c r="G41" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>